<commit_message>
Number  Array  code in java uploded
</commit_message>
<xml_diff>
--- a/LB_Program_Statements.xlsx
+++ b/LB_Program_Statements.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SHREYA\Desktop\LB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E5E1A271-F103-4AFA-AA96-6B288EC48261}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FC5F584-8331-4595-9769-30C4023903C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{529304FC-C76E-4A78-91F7-2381E30A6342}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="62">
   <si>
     <t>Jay Ganesh print in c</t>
   </si>
@@ -202,6 +202,24 @@
   </si>
   <si>
     <t>J 3 palindrome number with digits</t>
+  </si>
+  <si>
+    <t>C array basics for address</t>
+  </si>
+  <si>
+    <t>C Array size</t>
+  </si>
+  <si>
+    <t>C local array with member by member</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C global array with member by member </t>
+  </si>
+  <si>
+    <t>C sequence prnting array elements</t>
+  </si>
+  <si>
+    <t>C Iteration array printing</t>
   </si>
 </sst>
 </file>
@@ -553,7 +571,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A099BD82-CF9E-4D41-BD71-1A037607BD64}">
-  <dimension ref="A1:A93"/>
+  <dimension ref="A1:A99"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="49.85546875" bestFit="1" customWidth="1"/>
@@ -849,6 +867,36 @@
         <v>55</v>
       </c>
     </row>
+    <row r="94" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="95" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="96" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="97" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="98" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="99" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>61</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Number  Array Accepting IP in java uploded
</commit_message>
<xml_diff>
--- a/LB_Program_Statements.xlsx
+++ b/LB_Program_Statements.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SHREYA\Desktop\LB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FC5F584-8331-4595-9769-30C4023903C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9C7D9E0-2DC0-48DC-B76E-37FD1BDDF3F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{529304FC-C76E-4A78-91F7-2381E30A6342}"/>
   </bookViews>
@@ -219,7 +219,7 @@
     <t>C sequence prnting array elements</t>
   </si>
   <si>
-    <t>C Iteration array printing</t>
+    <t>C Iteration array printing static memory</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Number  Array Display(int * iPtr) in java uploded
</commit_message>
<xml_diff>
--- a/LB_Program_Statements.xlsx
+++ b/LB_Program_Statements.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SHREYA\Desktop\LB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9C7D9E0-2DC0-48DC-B76E-37FD1BDDF3F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DBC3753-FA4F-41D5-8CB4-06BDB11F667D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{529304FC-C76E-4A78-91F7-2381E30A6342}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="67">
   <si>
     <t>Jay Ganesh print in c</t>
   </si>
@@ -220,6 +220,21 @@
   </si>
   <si>
     <t>C Iteration array printing static memory</t>
+  </si>
+  <si>
+    <t>C Array ip op with sequence from user</t>
+  </si>
+  <si>
+    <t>C Array ip op with for loop from user</t>
+  </si>
+  <si>
+    <t>C function Callbyvalue</t>
+  </si>
+  <si>
+    <t>C  function call by address</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C Display(int * iPtr) for array </t>
   </si>
 </sst>
 </file>
@@ -571,7 +586,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A099BD82-CF9E-4D41-BD71-1A037607BD64}">
-  <dimension ref="A1:A99"/>
+  <dimension ref="A1:A104"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="49.85546875" bestFit="1" customWidth="1"/>
@@ -897,6 +912,31 @@
         <v>61</v>
       </c>
     </row>
+    <row r="100" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="101" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="102" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="103" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="104" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>66</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Number  Array taking ip from user in java uploded
</commit_message>
<xml_diff>
--- a/LB_Program_Statements.xlsx
+++ b/LB_Program_Statements.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SHREYA\Desktop\LB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DBC3753-FA4F-41D5-8CB4-06BDB11F667D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6625B068-0461-4CCC-ACF4-6557FD5FE156}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{529304FC-C76E-4A78-91F7-2381E30A6342}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="71">
   <si>
     <t>Jay Ganesh print in c</t>
   </si>
@@ -235,6 +235,18 @@
   </si>
   <si>
     <t xml:space="preserve">C Display(int * iPtr) for array </t>
+  </si>
+  <si>
+    <t xml:space="preserve">C </t>
+  </si>
+  <si>
+    <t>C Display array elements with function iteration</t>
+  </si>
+  <si>
+    <t>C Display(int Arr[], int iSize)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C Display() with ip elements form user </t>
   </si>
 </sst>
 </file>
@@ -586,7 +598,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A099BD82-CF9E-4D41-BD71-1A037607BD64}">
-  <dimension ref="A1:A104"/>
+  <dimension ref="A1:A117"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="49.85546875" bestFit="1" customWidth="1"/>
@@ -937,6 +949,26 @@
         <v>66</v>
       </c>
     </row>
+    <row r="106" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="110" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="114" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="117" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>70</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
summation of array elements in java uploded
</commit_message>
<xml_diff>
--- a/LB_Program_Statements.xlsx
+++ b/LB_Program_Statements.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SHREYA\Desktop\LB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6625B068-0461-4CCC-ACF4-6557FD5FE156}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34885674-AC60-4B77-850B-C20E41F932AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{529304FC-C76E-4A78-91F7-2381E30A6342}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="72">
   <si>
     <t>Jay Ganesh print in c</t>
   </si>
@@ -247,6 +247,9 @@
   </si>
   <si>
     <t xml:space="preserve">C Display() with ip elements form user </t>
+  </si>
+  <si>
+    <t>C Summation of all elements in array</t>
   </si>
 </sst>
 </file>
@@ -598,7 +601,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A099BD82-CF9E-4D41-BD71-1A037607BD64}">
-  <dimension ref="A1:A117"/>
+  <dimension ref="A1:A118"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="49.85546875" bestFit="1" customWidth="1"/>
@@ -969,6 +972,11 @@
         <v>70</v>
       </c>
     </row>
+    <row r="118" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>71</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
C program for even count
</commit_message>
<xml_diff>
--- a/LB_Program_Statements.xlsx
+++ b/LB_Program_Statements.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SHREYA\Desktop\LB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4BA3522-FF0A-4170-9B79-A81DFC87CFD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{390C073A-A04F-43DC-A0AD-89B2762D6519}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2205" yWindow="2205" windowWidth="21600" windowHeight="11295" xr2:uid="{529304FC-C76E-4A78-91F7-2381E30A6342}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="77">
   <si>
     <t>Jay Ganesh print in c</t>
   </si>
@@ -254,6 +254,9 @@
   </si>
   <si>
     <t>C Array memory allo with malloc</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> C dynamic array summation() same </t>
   </si>
 </sst>
 </file>
@@ -608,7 +611,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A099BD82-CF9E-4D41-BD71-1A037607BD64}">
-  <dimension ref="A1:A122"/>
+  <dimension ref="A1:A123"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="49.85546875" bestFit="1" customWidth="1"/>
@@ -1004,6 +1007,11 @@
         <v>72</v>
       </c>
     </row>
+    <row r="123" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>76</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
C program for even Summation
</commit_message>
<xml_diff>
--- a/LB_Program_Statements.xlsx
+++ b/LB_Program_Statements.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SHREYA\Desktop\LB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5783BC35-86E3-4EED-9BD4-80C91AF2615F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A06E345F-D123-42C9-8748-48122C0EC84A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2205" yWindow="2205" windowWidth="21600" windowHeight="11295" xr2:uid="{529304FC-C76E-4A78-91F7-2381E30A6342}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="79">
   <si>
     <t>Jay Ganesh print in c</t>
   </si>
@@ -260,6 +260,9 @@
   </si>
   <si>
     <t>C dynamic frequency of even no from array</t>
+  </si>
+  <si>
+    <t>C Summation of even nos from array</t>
   </si>
 </sst>
 </file>
@@ -614,7 +617,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A099BD82-CF9E-4D41-BD71-1A037607BD64}">
-  <dimension ref="A1:A124"/>
+  <dimension ref="A1:A125"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="49.85546875" bestFit="1" customWidth="1"/>
@@ -1020,6 +1023,11 @@
         <v>77</v>
       </c>
     </row>
+    <row r="125" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>78</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
C program for even odd
</commit_message>
<xml_diff>
--- a/LB_Program_Statements.xlsx
+++ b/LB_Program_Statements.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SHREYA\Desktop\LB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A06E345F-D123-42C9-8748-48122C0EC84A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82FAAAE1-B03B-4C1D-8BEE-357C35EF0FCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2205" yWindow="2205" windowWidth="21600" windowHeight="11295" xr2:uid="{529304FC-C76E-4A78-91F7-2381E30A6342}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="80">
   <si>
     <t>Jay Ganesh print in c</t>
   </si>
@@ -263,6 +263,9 @@
   </si>
   <si>
     <t>C Summation of even nos from array</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C frequency of odd nos </t>
   </si>
 </sst>
 </file>
@@ -617,7 +620,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A099BD82-CF9E-4D41-BD71-1A037607BD64}">
-  <dimension ref="A1:A125"/>
+  <dimension ref="A1:A126"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="49.85546875" bestFit="1" customWidth="1"/>
@@ -1028,6 +1031,11 @@
         <v>78</v>
       </c>
     </row>
+    <row r="126" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A126" t="s">
+        <v>79</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
C program for frequency of 11 in array
</commit_message>
<xml_diff>
--- a/LB_Program_Statements.xlsx
+++ b/LB_Program_Statements.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SHREYA\Desktop\LB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82FAAAE1-B03B-4C1D-8BEE-357C35EF0FCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{461ED829-696B-423B-8BF5-D06736AC12F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2205" yWindow="2205" windowWidth="21600" windowHeight="11295" xr2:uid="{529304FC-C76E-4A78-91F7-2381E30A6342}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="81">
   <si>
     <t>Jay Ganesh print in c</t>
   </si>
@@ -266,6 +266,9 @@
   </si>
   <si>
     <t xml:space="preserve">C frequency of odd nos </t>
+  </si>
+  <si>
+    <t>C count 11 occurance in array</t>
   </si>
 </sst>
 </file>
@@ -620,7 +623,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A099BD82-CF9E-4D41-BD71-1A037607BD64}">
-  <dimension ref="A1:A126"/>
+  <dimension ref="A1:A127"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="49.85546875" bestFit="1" customWidth="1"/>
@@ -1036,6 +1039,11 @@
         <v>79</v>
       </c>
     </row>
+    <row r="127" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A127" t="s">
+        <v>80</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
C program for if 11 present or not
</commit_message>
<xml_diff>
--- a/LB_Program_Statements.xlsx
+++ b/LB_Program_Statements.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SHREYA\Desktop\LB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{461ED829-696B-423B-8BF5-D06736AC12F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5ACD77BF-2914-42DC-B97E-DEB73B194155}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2205" yWindow="2205" windowWidth="21600" windowHeight="11295" xr2:uid="{529304FC-C76E-4A78-91F7-2381E30A6342}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="83">
   <si>
     <t>Jay Ganesh print in c</t>
   </si>
@@ -269,6 +269,12 @@
   </si>
   <si>
     <t>C count 11 occurance in array</t>
+  </si>
+  <si>
+    <t>C if 11 present or not true or false bad progra</t>
+  </si>
+  <si>
+    <t>C 11 present or not with flag mediam good</t>
   </si>
 </sst>
 </file>
@@ -623,7 +629,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A099BD82-CF9E-4D41-BD71-1A037607BD64}">
-  <dimension ref="A1:A127"/>
+  <dimension ref="A1:A129"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="49.85546875" bestFit="1" customWidth="1"/>
@@ -1044,6 +1050,16 @@
         <v>80</v>
       </c>
     </row>
+    <row r="128" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A128" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="129" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A129" t="s">
+        <v>82</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
C program for if NO present or not
</commit_message>
<xml_diff>
--- a/LB_Program_Statements.xlsx
+++ b/LB_Program_Statements.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SHREYA\Desktop\LB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5ACD77BF-2914-42DC-B97E-DEB73B194155}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08476B4A-8DA6-44CE-899C-E020E7083119}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2205" yWindow="2205" windowWidth="21600" windowHeight="11295" xr2:uid="{529304FC-C76E-4A78-91F7-2381E30A6342}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="84">
   <si>
     <t>Jay Ganesh print in c</t>
   </si>
@@ -275,6 +275,9 @@
   </si>
   <si>
     <t>C 11 present or not with flag mediam good</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C if iNo is present in array entered by user </t>
   </si>
 </sst>
 </file>
@@ -629,7 +632,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A099BD82-CF9E-4D41-BD71-1A037607BD64}">
-  <dimension ref="A1:A129"/>
+  <dimension ref="A1:A130"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="49.85546875" bestFit="1" customWidth="1"/>
@@ -1060,6 +1063,11 @@
         <v>82</v>
       </c>
     </row>
+    <row r="130" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A130" t="s">
+        <v>83</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
C program for if NO present or not without flag
</commit_message>
<xml_diff>
--- a/LB_Program_Statements.xlsx
+++ b/LB_Program_Statements.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SHREYA\Desktop\LB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08476B4A-8DA6-44CE-899C-E020E7083119}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D7D3985-4AC2-4448-AD5D-4A3B3D8DE9D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2205" yWindow="2205" windowWidth="21600" windowHeight="11295" xr2:uid="{529304FC-C76E-4A78-91F7-2381E30A6342}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="87">
   <si>
     <t>Jay Ganesh print in c</t>
   </si>
@@ -277,7 +277,16 @@
     <t>C 11 present or not with flag mediam good</t>
   </si>
   <si>
-    <t xml:space="preserve">C if iNo is present in array entered by user </t>
+    <t>C if iNo is present in array entered by user without flag</t>
+  </si>
+  <si>
+    <t>C if iNo is present in array entered by user with flag</t>
+  </si>
+  <si>
+    <t>C if iNo is present in array entered by user without flag but new variable int</t>
+  </si>
+  <si>
+    <t>C if iNo is present in array entered by user without flag without creating new variable bestt</t>
   </si>
 </sst>
 </file>
@@ -632,10 +641,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A099BD82-CF9E-4D41-BD71-1A037607BD64}">
-  <dimension ref="A1:A130"/>
+  <dimension ref="A1:A134"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="49.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="83.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -1065,7 +1074,27 @@
     </row>
     <row r="130" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="131" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A131" t="s">
         <v>83</v>
+      </c>
+    </row>
+    <row r="132" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A132" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="133" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A133" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="134" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A134" t="s">
+        <v>86</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
C program for maximum and minimum from array
</commit_message>
<xml_diff>
--- a/LB_Program_Statements.xlsx
+++ b/LB_Program_Statements.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SHREYA\Desktop\LB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D7D3985-4AC2-4448-AD5D-4A3B3D8DE9D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C18B02D7-3A55-461D-9226-D5BFAB83B2C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2205" yWindow="2205" windowWidth="21600" windowHeight="11295" xr2:uid="{529304FC-C76E-4A78-91F7-2381E30A6342}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="89">
   <si>
     <t>Jay Ganesh print in c</t>
   </si>
@@ -287,6 +287,12 @@
   </si>
   <si>
     <t>C if iNo is present in array entered by user without flag without creating new variable bestt</t>
+  </si>
+  <si>
+    <t>C maximum from array</t>
+  </si>
+  <si>
+    <t>C minimum from array</t>
   </si>
 </sst>
 </file>
@@ -641,7 +647,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A099BD82-CF9E-4D41-BD71-1A037607BD64}">
-  <dimension ref="A1:A134"/>
+  <dimension ref="A1:A136"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="83.7109375" bestFit="1" customWidth="1"/>
@@ -1097,6 +1103,16 @@
         <v>86</v>
       </c>
     </row>
+    <row r="135" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A135" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="136" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A136" t="s">
+        <v>88</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
program in java for array
</commit_message>
<xml_diff>
--- a/LB_Program_Statements.xlsx
+++ b/LB_Program_Statements.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SHREYA\Desktop\LB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C18B02D7-3A55-461D-9226-D5BFAB83B2C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B83E8E83-36FE-42D6-8123-7E235A4D47F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2205" yWindow="2205" windowWidth="21600" windowHeight="11295" xr2:uid="{529304FC-C76E-4A78-91F7-2381E30A6342}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="96">
   <si>
     <t>Jay Ganesh print in c</t>
   </si>
@@ -293,6 +293,27 @@
   </si>
   <si>
     <t>C minimum from array</t>
+  </si>
+  <si>
+    <t>java Array with sequence</t>
+  </si>
+  <si>
+    <t>java Array with iteration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">java for(int iCnt in loop </t>
+  </si>
+  <si>
+    <t>java for(int iCnt  in loop accessing it outside loop error</t>
+  </si>
+  <si>
+    <t>java array creation with new and display elements</t>
+  </si>
+  <si>
+    <t xml:space="preserve">java gc free the memory </t>
+  </si>
+  <si>
+    <t>J2 summation function in main</t>
   </si>
 </sst>
 </file>
@@ -647,7 +668,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A099BD82-CF9E-4D41-BD71-1A037607BD64}">
-  <dimension ref="A1:A136"/>
+  <dimension ref="A1:A143"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="83.7109375" bestFit="1" customWidth="1"/>
@@ -1113,6 +1134,41 @@
         <v>88</v>
       </c>
     </row>
+    <row r="137" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A137" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="138" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A138" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="139" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A139" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="140" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A140" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="141" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A141" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="142" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A142" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="143" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A143" t="s">
+        <v>95</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
code for oop and sequential pattern printing uploded
</commit_message>
<xml_diff>
--- a/LB_Program_Statements.xlsx
+++ b/LB_Program_Statements.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SHREYA\Desktop\LB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B83E8E83-36FE-42D6-8123-7E235A4D47F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A35609D-13E5-4882-93A0-84366F361B72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2205" yWindow="2205" windowWidth="21600" windowHeight="11295" xr2:uid="{529304FC-C76E-4A78-91F7-2381E30A6342}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{529304FC-C76E-4A78-91F7-2381E30A6342}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="145">
   <si>
     <t>Jay Ganesh print in c</t>
   </si>
@@ -314,6 +314,169 @@
   </si>
   <si>
     <t>J2 summation function in main</t>
+  </si>
+  <si>
+    <t>C update of elements call by address</t>
+  </si>
+  <si>
+    <t>j2 update of elements of array even address is not there as it's call by reference</t>
+  </si>
+  <si>
+    <t>J3 update of elements of array even address is not there as it's call by reference with static Update</t>
+  </si>
+  <si>
+    <t>J3 update of elements of array even address is not there as it's call by reference without static Update</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>CPP</t>
+  </si>
+  <si>
+    <t>JAVA</t>
+  </si>
+  <si>
+    <t>Java</t>
+  </si>
+  <si>
+    <t>CPP Array Display</t>
+  </si>
+  <si>
+    <t>Cpp</t>
+  </si>
+  <si>
+    <t>Dyanamic memory allocation of array in cpp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Summation function </t>
+  </si>
+  <si>
+    <t>N number in array and summation of all oop concept</t>
+  </si>
+  <si>
+    <t>printing linear * on screen in line from number from user J1</t>
+  </si>
+  <si>
+    <t>java</t>
+  </si>
+  <si>
+    <t>1  2  3  4  5 printing from user input j1</t>
+  </si>
+  <si>
+    <t>1 * 2 * 3 * 4 * 5 *</t>
+  </si>
+  <si>
+    <t>* # * # * # * # * #</t>
+  </si>
+  <si>
+    <t>*1* *2* *3* *4* *5*</t>
+  </si>
+  <si>
+    <t>1  *  3  *  5  *  7</t>
+  </si>
+  <si>
+    <t>1  *  2  *  3  *  4  when 1p = 7 with iCount veriable</t>
+  </si>
+  <si>
+    <t>1  *  2  *  3  *  4  when 1p = 7 without iCount veriable iCnt/2 + 1 for odd</t>
+  </si>
+  <si>
+    <t>float la ++ nahi chlat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a  b  c  d  e  f  g when user input number </t>
+  </si>
+  <si>
+    <t>a  b  c  d  e  f  g using (iCnt = 1, ch = 'a'; iCnt &lt;= iNo; iCnt++, ch++) in a single line</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a  b  c  d  e  f  g using (iCnt = 1, ch = 97; iCnt &lt;= iNo; iCnt++, ch++) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">a  b  c  d  e  f  g using (iCnt = 1, ch = 65; iCnt &lt;= iNo; iCnt++, ch++) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">a  b  c  d  e  f  g using (iCnt = 1, ch = 'A'; iCnt &lt;= iNo; iCnt++, ch++) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">A  *  B  *  C  *  D  </t>
+  </si>
+  <si>
+    <t>A  *  C  *  E  *  G</t>
+  </si>
+  <si>
+    <t>A  2  C  4  E  6 G</t>
+  </si>
+  <si>
+    <t>A  b  C  d  E  f  G with two ch1 and ch2</t>
+  </si>
+  <si>
+    <t>48 = 0 ;65 = A ;97 = a</t>
+  </si>
+  <si>
+    <t>*  *  *  #  #  #  *  *  *  #  #   for 11</t>
+  </si>
+  <si>
+    <t>* * * * 
+* * * *
+* * * *  user input</t>
+  </si>
+  <si>
+    <t>* * * * 
+* * * *
+* * * * hardcoded</t>
+  </si>
+  <si>
+    <t>* * * * with sequence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1  2  3  4
+1  2  3  4 
+1  2  3  4 
+1  2  3  4    from user </t>
+  </si>
+  <si>
+    <t xml:space="preserve">*  *  *  * 
+$  $  $  $
+*  *  *  * 
+$  $  $  $ </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1  1  1  1 
+2  2  2  2
+3  3  3  3
+4  4  4  4 </t>
+  </si>
+  <si>
+    <t>Error summation function for array as default access specifier for function is private</t>
+  </si>
+  <si>
+    <t>public int summation()</t>
+  </si>
+  <si>
+    <t>size of object having pointer for array is 16 with padding 4</t>
+  </si>
+  <si>
+    <t>added pragma pack 1 for no padding</t>
+  </si>
+  <si>
+    <t>error due to no default constuctor</t>
+  </si>
+  <si>
+    <t>code with default constructor</t>
+  </si>
+  <si>
+    <t>2 constructor parametrized and default</t>
+  </si>
+  <si>
+    <t>good oop programming with class and constructors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#  &amp;  #  &amp;
+#  &amp;  #  &amp;
+#  &amp;  #  &amp;
+#  &amp;  #  &amp; </t>
   </si>
 </sst>
 </file>
@@ -349,11 +512,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -668,505 +832,1108 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A099BD82-CF9E-4D41-BD71-1A037607BD64}">
-  <dimension ref="A1:A143"/>
+  <dimension ref="A1:C196"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="83.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="93.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B17" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B18" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B19" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B24" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B25" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B27" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B28" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B33" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B34" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B35" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B36" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B37" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B39" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B40" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B46" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B48" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B50" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B52" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B53" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B57" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B59" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B60" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B61" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B62" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B63" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B64" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B65" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B69" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B70" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B72" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B73" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B74" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B75" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B76" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B77" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B79" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B81" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="84" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B83" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="85" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B84" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="86" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B85" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="87" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B86" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B87" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="89" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B88" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="90" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B89" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B90" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="92" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B91" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="93" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B92" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="94" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B93" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="95" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B94" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="96" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B95" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B96" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="98" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B97" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="99" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B98" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="100" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B99" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="101" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B100" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="102" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B101" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="103" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B102" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="104" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B103" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="105" spans="1:1" ht="30" x14ac:dyDescent="0.25">
+      <c r="B104" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A105" s="1" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="106" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B105" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="106" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="110" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B106" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="114" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B110" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="114" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="117" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B114" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="118" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B117" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="118" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="119" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B118" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="119" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="120" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B119" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="120" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="122" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B120" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="122" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="123" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B122" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="123" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="124" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B123" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="124" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="125" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B124" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="125" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="126" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B125" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="126" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="127" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B126" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="127" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="128" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B127" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="128" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="129" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B128" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="129" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="130" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B129" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="130" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="131" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B130" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="131" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="132" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B131" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="132" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="133" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B132" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="133" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="134" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B133" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="134" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="135" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B134" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="135" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="136" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B135" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="136" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="137" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B136" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="137" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="138" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B137" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="138" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="139" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B138" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="139" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="140" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B139" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="140" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="141" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B140" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="141" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="142" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B141" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="142" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="143" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B142" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="143" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>95</v>
+      </c>
+      <c r="B143" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="144" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A144" t="s">
+        <v>96</v>
+      </c>
+      <c r="B144" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="145" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A145" t="s">
+        <v>97</v>
+      </c>
+      <c r="B145" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="146" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A146" t="s">
+        <v>98</v>
+      </c>
+      <c r="B146" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="147" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A147" t="s">
+        <v>99</v>
+      </c>
+      <c r="B147" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="148" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A148" t="s">
+        <v>104</v>
+      </c>
+      <c r="B148" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="149" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A149" t="s">
+        <v>106</v>
+      </c>
+      <c r="B149" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="150" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A150" t="s">
+        <v>107</v>
+      </c>
+      <c r="B150" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="151" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A151" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="152" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A152" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="153" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A153" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="154" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A154" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="155" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A155" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="156" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A156" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="157" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A157" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="158" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A158" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="169" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A169" t="s">
+        <v>108</v>
+      </c>
+      <c r="B169" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="171" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A171" t="s">
+        <v>109</v>
+      </c>
+      <c r="B171" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="172" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A172" t="s">
+        <v>111</v>
+      </c>
+      <c r="B172" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="173" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A173" t="s">
+        <v>112</v>
+      </c>
+      <c r="B173" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="174" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A174" t="s">
+        <v>113</v>
+      </c>
+      <c r="B174" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="175" spans="1:2" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A175" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="B175" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="176" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A176" t="s">
+        <v>115</v>
+      </c>
+      <c r="B176" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="177" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A177" t="s">
+        <v>116</v>
+      </c>
+      <c r="B177" t="s">
+        <v>110</v>
+      </c>
+      <c r="C177" s="2"/>
+    </row>
+    <row r="178" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A178" t="s">
+        <v>117</v>
+      </c>
+      <c r="B178" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="179" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A179" t="s">
+        <v>119</v>
+      </c>
+      <c r="B179" t="s">
+        <v>110</v>
+      </c>
+      <c r="C179" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="180" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A180" t="s">
+        <v>120</v>
+      </c>
+      <c r="B180" t="s">
+        <v>110</v>
+      </c>
+      <c r="C180" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="181" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A181" t="s">
+        <v>121</v>
+      </c>
+      <c r="B181" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="182" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A182" t="s">
+        <v>122</v>
+      </c>
+      <c r="B182" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="183" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A183" t="s">
+        <v>123</v>
+      </c>
+      <c r="B183" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="184" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A184" t="s">
+        <v>124</v>
+      </c>
+      <c r="B184" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="185" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A185" t="s">
+        <v>125</v>
+      </c>
+      <c r="B185" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="186" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A186" t="s">
+        <v>126</v>
+      </c>
+      <c r="B186" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="187" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A187" t="s">
+        <v>127</v>
+      </c>
+      <c r="B187" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="188" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A188" t="s">
+        <v>129</v>
+      </c>
+      <c r="B188" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="189" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A189" t="s">
+        <v>132</v>
+      </c>
+      <c r="B189" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="191" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A191" s="1" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="192" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A192" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="B192" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="193" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+      <c r="A193" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B193" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="194" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+      <c r="A194" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="B194" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="195" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+      <c r="A195" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="B195" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="196" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+      <c r="A196" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="B196" t="s">
+        <v>110</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
program 197 in java for pattern added
</commit_message>
<xml_diff>
--- a/LB_Program_Statements.xlsx
+++ b/LB_Program_Statements.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SHREYA\Desktop\LB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A35609D-13E5-4882-93A0-84366F361B72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BA34BC6-52FE-483E-B0D2-1661A2049F31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{529304FC-C76E-4A78-91F7-2381E30A6342}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{529304FC-C76E-4A78-91F7-2381E30A6342}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="147">
   <si>
     <t>Jay Ganesh print in c</t>
   </si>
@@ -477,6 +477,15 @@
 #  &amp;  #  &amp;
 #  &amp;  #  &amp;
 #  &amp;  #  &amp; </t>
+  </si>
+  <si>
+    <t>TC = O(N^2)</t>
+  </si>
+  <si>
+    <t>$  $  $  $
+$  $  $  $
+$  $  $  $
+$  $  $  $</t>
   </si>
 </sst>
 </file>
@@ -832,7 +841,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A099BD82-CF9E-4D41-BD71-1A037607BD64}">
-  <dimension ref="A1:C196"/>
+  <dimension ref="A1:C197"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="93.140625" bestFit="1" customWidth="1"/>
@@ -1904,7 +1913,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="193" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:3" ht="60" x14ac:dyDescent="0.25">
       <c r="A193" s="1" t="s">
         <v>133</v>
       </c>
@@ -1912,7 +1921,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="194" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:3" ht="60" x14ac:dyDescent="0.25">
       <c r="A194" s="1" t="s">
         <v>135</v>
       </c>
@@ -1920,7 +1929,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="195" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:3" ht="60" x14ac:dyDescent="0.25">
       <c r="A195" s="1" t="s">
         <v>134</v>
       </c>
@@ -1928,11 +1937,22 @@
         <v>110</v>
       </c>
     </row>
-    <row r="196" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:3" ht="60" x14ac:dyDescent="0.25">
       <c r="A196" s="1" t="s">
         <v>144</v>
       </c>
       <c r="B196" t="s">
+        <v>110</v>
+      </c>
+      <c r="C196" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="197" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="A197" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="B197" t="s">
         <v>110</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Codes from 197 to 230 is uploded
</commit_message>
<xml_diff>
--- a/LB_Program_Statements.xlsx
+++ b/LB_Program_Statements.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SHREYA\Desktop\LB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BA34BC6-52FE-483E-B0D2-1661A2049F31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF533B8B-22E1-4662-AEC0-4A1EC72ACFEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{529304FC-C76E-4A78-91F7-2381E30A6342}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="181">
   <si>
     <t>Jay Ganesh print in c</t>
   </si>
@@ -486,6 +486,223 @@
 $  $  $  $
 $  $  $  $
 $  $  $  $</t>
+  </si>
+  <si>
+    <t>Homogeneous nesting</t>
+  </si>
+  <si>
+    <t>1  1  1  1
+2  2  2  2
+3  3  3  3
+4  4  4  4</t>
+  </si>
+  <si>
+    <t>1  2  3  4  
+1  2  3  4
+1  2  3  4
+1  2  3  4</t>
+  </si>
+  <si>
+    <t>$  $  $  $
+#  #  #  #
+$  $  $  $
+#  #  #  #</t>
+  </si>
+  <si>
+    <t>$  $  $  $
+#  #  #  #
+$  $  $  $
+#  #  #  #
+by reducing if else</t>
+  </si>
+  <si>
+    <t>$  $  $  $
+#  #  #  #
+$  $  $  $
+#  #  #  #
+without using if else with char array</t>
+  </si>
+  <si>
+    <t>A  B  C  D
+A  B  C  D
+A  B  C  D
+A  B  C  D</t>
+  </si>
+  <si>
+    <t>a  b  c  d 
+a  b  c  d
+a  b  c  d
+a  b  c  d</t>
+  </si>
+  <si>
+    <t>a  b  c  d 
+a  b  c  d
+a  b  c  d
+a  b  c  d using ascii value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a  b  c  d 
+1  2  3  4
+a  b  c  d
+1  2  3  4 </t>
+  </si>
+  <si>
+    <t>4  4  4  4
+3  3  3  3
+2  2  2  2
+1  1  1  1 with another veriable</t>
+  </si>
+  <si>
+    <t>4  4  4  4
+3  3  3  3
+2  2  2  2
+1  1  1  1  by reversing the outer loop</t>
+  </si>
+  <si>
+    <t>$  @  @  @
+@  $  @  @
+@  @  $  @
+@  @  @  $
+with invalid conition for diagonal</t>
+  </si>
+  <si>
+    <t>%  @  @  @  @  %
+%  @  @  @  @  %
+%  @  @  @  @  %
+%  @  @  @  @  %
+%  @  @  @  @  %
+%  @  @  @  @  %</t>
+  </si>
+  <si>
+    <t>in c we must use %% two times for printing single %</t>
+  </si>
+  <si>
+    <t>%  %  %  %  %  %
+%  @  @  @  @  %
+%  @  @  @  @  %
+%  @  @  @  @  %
+%  @  @  @  @  %
+%  %  %  %  %  %</t>
+  </si>
+  <si>
+    <t>%  %  %  %  %  %
+%                     %
+%                     %
+%                    %
+%                    %
+%  %  %  %  %  %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">%  #  #  #
+%  %  #  #
+%  %  %  #
+%  %  %  % </t>
+  </si>
+  <si>
+    <t>* 
+*  *  
+*  *  *  
+*  *  *  *   
+optimized reduced loop printing
+TC &gt;O(N^2/2)</t>
+  </si>
+  <si>
+    <t>1
+1  2
+1  2  3
+1  2  3  4</t>
+  </si>
+  <si>
+    <t>a
+a  b
+a  b  c
+a  b  c  d</t>
+  </si>
+  <si>
+    <t>a
+b  b  
+c  c  c  
+d  d  d  d</t>
+  </si>
+  <si>
+    <t>a
+b  c  
+d  e  f  
+g  h  i  j</t>
+  </si>
+  <si>
+    <t>*
+*  *
+*  $  *
+*  $  $  *
+*  $  $  $  *
+*  *  *  *  *  *</t>
+  </si>
+  <si>
+    <t>*
+*  *
+*      *
+*          *
+*              *
+*  *  *  *  *  *</t>
+  </si>
+  <si>
+    <t xml:space="preserve">instruction queue madhe if else vadhala ki vel vadhato </t>
+  </si>
+  <si>
+    <t xml:space="preserve">* * * * 
+* * * *
+* * * * sequencial for loop </t>
+  </si>
+  <si>
+    <t>$  @  @  @
+@  $  @  @
+@  @  $  @
+@  @  @  $
+with backward outer loop</t>
+  </si>
+  <si>
+    <t>$  @  @  @
+@  $  @  @
+@  @  $  @
+@  @  @  $
+with forward loop</t>
+  </si>
+  <si>
+    <t>#    #    #    #    #    #
+@  @  @  @  @  @
+@  @  @  @  @  @
+@  @  @  @  @  @
+@  @  @  @  @  @
+#    #    #    #    #   #</t>
+  </si>
+  <si>
+    <t>%  %  %  %  %  %
+%                      %
+%                      %
+%                      %
+%                      %
+%  %  %  %  %  %</t>
+  </si>
+  <si>
+    <t>%  %  %  %  %  %
+%  %                  %
+%        %            %
+%             %       %
+%                  %  %
+%  %  %  %  %  %</t>
+  </si>
+  <si>
+    <t>* 
+*  *  
+*  *  *  
+*  *  *  * (i&gt;=j)</t>
+  </si>
+  <si>
+    <t>* 
+*  *  
+*  *  *  
+*  *  *  * (j&lt;=i)</t>
   </si>
 </sst>
 </file>
@@ -521,12 +738,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -841,11 +1061,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A099BD82-CF9E-4D41-BD71-1A037607BD64}">
-  <dimension ref="A1:C197"/>
+  <dimension ref="A1:C229"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="93.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.85546875" customWidth="1"/>
+    <col min="3" max="3" width="48.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -1900,6 +2120,14 @@
         <v>110</v>
       </c>
     </row>
+    <row r="190" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A190" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="B190" t="s">
+        <v>110</v>
+      </c>
+    </row>
     <row r="191" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A191" s="1" t="s">
         <v>131</v>
@@ -1953,6 +2181,246 @@
         <v>146</v>
       </c>
       <c r="B197" t="s">
+        <v>110</v>
+      </c>
+      <c r="C197" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="198" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="A198" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="B198" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="199" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="A199" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="B199" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="200" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="A200" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="B200" t="s">
+        <v>110</v>
+      </c>
+      <c r="C200" s="1" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="201" spans="1:3" ht="75" x14ac:dyDescent="0.25">
+      <c r="A201" s="1" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="202" spans="1:3" ht="90" x14ac:dyDescent="0.25">
+      <c r="A202" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="B202" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="203" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="A203" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="B203" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="204" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="A204" s="1" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="205" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="A205" s="1" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="206" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="A206" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="B206" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="207" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="A207" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="B207" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="208" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="A208" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="B208" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="209" spans="1:3" ht="75" x14ac:dyDescent="0.25">
+      <c r="A209" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="B209" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="210" spans="1:3" ht="75" x14ac:dyDescent="0.25">
+      <c r="A210" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="B210" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="211" spans="1:3" ht="75" x14ac:dyDescent="0.25">
+      <c r="A211" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="B211" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="212" spans="1:3" ht="90" x14ac:dyDescent="0.25">
+      <c r="A212" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="B212" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="213" spans="1:3" ht="90" x14ac:dyDescent="0.25">
+      <c r="A213" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="B213" t="s">
+        <v>110</v>
+      </c>
+      <c r="C213" s="3" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="214" spans="1:3" ht="90" x14ac:dyDescent="0.25">
+      <c r="A214" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="B214" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="215" spans="1:3" ht="90" x14ac:dyDescent="0.25">
+      <c r="A215" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="B215" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="216" spans="1:3" ht="90" x14ac:dyDescent="0.25">
+      <c r="A216" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="B216" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="217" spans="1:3" ht="90" x14ac:dyDescent="0.25">
+      <c r="A217" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="B217" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="218" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="A218" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="B218" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="221" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="A221" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="B221" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="222" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="A222" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="B222" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="223" spans="1:3" ht="90" x14ac:dyDescent="0.25">
+      <c r="A223" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="B223" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="224" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="A224" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="B224" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="225" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+      <c r="A225" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="B225" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="226" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+      <c r="A226" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="B226" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="227" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+      <c r="A227" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="B227" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="228" spans="1:2" ht="90" x14ac:dyDescent="0.25">
+      <c r="A228" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="B228" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="229" spans="1:2" ht="90" x14ac:dyDescent="0.25">
+      <c r="A229" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="B229" t="s">
         <v>110</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Codes on biwise operator uploded
</commit_message>
<xml_diff>
--- a/LB_Program_Statements.xlsx
+++ b/LB_Program_Statements.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SHREYA\Desktop\LB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A223B44-FE26-455A-B592-390491DB79CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2C0851E-707D-4773-B26F-290B8AC85B04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2205" yWindow="2205" windowWidth="21600" windowHeight="11295" xr2:uid="{529304FC-C76E-4A78-91F7-2381E30A6342}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{529304FC-C76E-4A78-91F7-2381E30A6342}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="388" uniqueCount="212">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="481" uniqueCount="259">
   <si>
     <t>Jay Ganesh print in c</t>
   </si>
@@ -801,6 +801,163 @@
   </si>
   <si>
     <t>count frequency of capital char in string</t>
+  </si>
+  <si>
+    <t>short circuit evaluation will not check second cond in &amp;&amp; if first cond is false</t>
+  </si>
+  <si>
+    <t>count frequency of small and capital letter in string</t>
+  </si>
+  <si>
+    <t>char Arr[] = str.toCharArray(); reduced the call of charAt() as it was called double the size of string</t>
+  </si>
+  <si>
+    <t>String is immutable so convert it to char array for updation</t>
+  </si>
+  <si>
+    <t>Count Digits in string</t>
+  </si>
+  <si>
+    <t>Count of Spaces in string</t>
+  </si>
+  <si>
+    <t>Count Frequency of special symbols in string</t>
+  </si>
+  <si>
+    <t>|| will check firsr cond if its true it will not check second cond goes in</t>
+  </si>
+  <si>
+    <t>error due to not importing package</t>
+  </si>
+  <si>
+    <t>replace a or A to _ using sting to array then array to string = String ret = new String(Arr);</t>
+  </si>
+  <si>
+    <t>return new String(Arr) without creating extra string</t>
+  </si>
+  <si>
+    <t>to upper string error dut to uncompatible datatype int to char</t>
+  </si>
+  <si>
+    <t>to upper case in string error due to not putting if condition</t>
+  </si>
+  <si>
+    <t xml:space="preserve">to upper case in string </t>
+  </si>
+  <si>
+    <t>to upper and to lower</t>
+  </si>
+  <si>
+    <t>Toggle issue due to if else (not using else if)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Toggle cases code </t>
+  </si>
+  <si>
+    <t>Reverse display issue due to str at \0</t>
+  </si>
+  <si>
+    <t>reverse display of string by adding str--</t>
+  </si>
+  <si>
+    <t>o
+lo
+llo
+ello
+Hello</t>
+  </si>
+  <si>
+    <t>reverse in one line</t>
+  </si>
+  <si>
+    <t>PP</t>
+  </si>
+  <si>
+    <t>ArrayX *aobj1 = new ArrayX(5);</t>
+  </si>
+  <si>
+    <t>static memory allocation for object</t>
+  </si>
+  <si>
+    <t>reverse String in the same string by address   TC = O(2N)
+without = in start end condition</t>
+  </si>
+  <si>
+    <t>reverse String in the same string by address   TC = O(2N)
+with = in start end condition</t>
+  </si>
+  <si>
+    <t>Call by address
+void swap(int *ptr1, int *ptr2)</t>
+  </si>
+  <si>
+    <t>Call by value
+void swap(int No1, int No2)</t>
+  </si>
+  <si>
+    <t>swap in main using temp</t>
+  </si>
+  <si>
+    <t>Decimal, Ocatal and hexadecimal of a integer</t>
+  </si>
+  <si>
+    <t>Decimal, Ocatal and hexadecimal of a integer of 197</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Decimal to Binary using while loop like digit but % 2 and / 2 </t>
+  </si>
+  <si>
+    <t>AND operation on decimal &amp;</t>
+  </si>
+  <si>
+    <t>Decimal AND Decimal
+Decimal OR Decimal
+Decimal XOR Decimal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">with using while loop and converting to binary not good </t>
+  </si>
+  <si>
+    <t>accept number and count number of 1 in binary using if in while</t>
+  </si>
+  <si>
+    <t>accept number and check whether 3rd bit is on or off</t>
+  </si>
+  <si>
+    <t>accept number and check whether 3rd bit is on or off but variables are unsigned</t>
+  </si>
+  <si>
+    <t xml:space="preserve">accept number and check whether 3rd bit is on or off but variables are unsigned using typedef UINT
+ </t>
+  </si>
+  <si>
+    <t>accept number and check whether 7rd bit 
+is on or off but variables are unsigned using typedef</t>
+  </si>
+  <si>
+    <t>2 ^ 7 = 64 so &amp; 64</t>
+  </si>
+  <si>
+    <t>accept number and check whether 13rd bit 
+is on or off but variables are unsigned using typedef</t>
+  </si>
+  <si>
+    <t>13 th bit 4096</t>
+  </si>
+  <si>
+    <t>accept number and check whether 17rth bit 
+is on or off but variables are unsigned using typedef and iMask is in hexadecimal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x00010000 = 0x10000 so remove 0 from start </t>
+  </si>
+  <si>
+    <t>0x00010000  will tell 17th bit (static mask desgining)</t>
+  </si>
+  <si>
+    <t>accept number and position to check from user
+do iMask = 0x1
+then iMask &lt;&lt; (iPos - 1)</t>
   </si>
 </sst>
 </file>
@@ -1159,11 +1316,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A099BD82-CF9E-4D41-BD71-1A037607BD64}">
-  <dimension ref="A1:C270"/>
+  <dimension ref="A1:C317"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="93.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="61.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="69.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -1963,7 +2120,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="145" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
         <v>97</v>
       </c>
@@ -1971,7 +2128,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="146" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
         <v>98</v>
       </c>
@@ -1979,7 +2136,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="147" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
         <v>99</v>
       </c>
@@ -1987,7 +2144,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="148" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
         <v>104</v>
       </c>
@@ -1995,7 +2152,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="149" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
         <v>106</v>
       </c>
@@ -2003,7 +2160,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="150" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
         <v>107</v>
       </c>
@@ -2011,44 +2168,114 @@
         <v>101</v>
       </c>
     </row>
-    <row r="151" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="152" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B151" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="152" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="153" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B152" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="153" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="154" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B153" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="154" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="155" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B154" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="155" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="156" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B155" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="156" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="157" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B156" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="157" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="158" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B157" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="158" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
         <v>143</v>
+      </c>
+      <c r="B158" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="159" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A159" t="s">
+        <v>234</v>
+      </c>
+      <c r="B159" t="s">
+        <v>101</v>
+      </c>
+      <c r="C159" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="160" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B160" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="161" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B161" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="162" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B162" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="163" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B163" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="164" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B164" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="165" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B165" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="166" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B166" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="169" spans="1:2" x14ac:dyDescent="0.25">
@@ -2717,6 +2944,305 @@
       </c>
       <c r="B270" t="s">
         <v>110</v>
+      </c>
+      <c r="C270" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="271" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A271" t="s">
+        <v>213</v>
+      </c>
+      <c r="B271" t="s">
+        <v>110</v>
+      </c>
+      <c r="C271" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="272" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A272" t="s">
+        <v>214</v>
+      </c>
+      <c r="B272" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="273" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A273" t="s">
+        <v>216</v>
+      </c>
+      <c r="B273" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="274" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A274" t="s">
+        <v>217</v>
+      </c>
+      <c r="B274" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="275" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A275" t="s">
+        <v>218</v>
+      </c>
+      <c r="B275" t="s">
+        <v>110</v>
+      </c>
+      <c r="C275" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="276" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A276" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="278" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A278" t="s">
+        <v>221</v>
+      </c>
+      <c r="B278" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="279" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A279" t="s">
+        <v>222</v>
+      </c>
+      <c r="B279" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="281" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A281" t="s">
+        <v>223</v>
+      </c>
+      <c r="B281" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="285" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A285" t="s">
+        <v>224</v>
+      </c>
+      <c r="B285" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="286" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A286" t="s">
+        <v>225</v>
+      </c>
+      <c r="B286" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="287" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A287" t="s">
+        <v>226</v>
+      </c>
+      <c r="B287" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="288" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A288" t="s">
+        <v>227</v>
+      </c>
+      <c r="B288" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="289" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A289" t="s">
+        <v>228</v>
+      </c>
+      <c r="B289" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="291" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A291" t="s">
+        <v>229</v>
+      </c>
+      <c r="B291" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="292" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A292" t="s">
+        <v>230</v>
+      </c>
+      <c r="B292" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="293" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A293" t="s">
+        <v>232</v>
+      </c>
+      <c r="B293" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="294" spans="1:2" ht="75" x14ac:dyDescent="0.25">
+      <c r="A294" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="B294" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="296" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A296" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="297" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A297" s="1" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="298" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A298" s="1" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="299" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A299" s="1" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="300" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A300" s="1" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="301" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A301" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="B301" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="302" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A302" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="B302" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="303" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A303" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="B303" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="304" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A304" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B304" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="305" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A305" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="B305" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="306" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A306" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="B306" t="s">
+        <v>100</v>
+      </c>
+      <c r="C306" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="308" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A308" s="1" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="309" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A309" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="B309" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="310" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A310" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="B310" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="311" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A311" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="B311" t="s">
+        <v>100</v>
+      </c>
+      <c r="C311" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="312" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A312" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="B312" t="s">
+        <v>100</v>
+      </c>
+      <c r="C312" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="313" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A313" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="B313" t="s">
+        <v>100</v>
+      </c>
+      <c r="C313" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="314" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A314" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="B314" t="s">
+        <v>100</v>
+      </c>
+      <c r="C314" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="317" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A317" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="B317" t="s">
+        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Codes on biwise Operator for manual shift
</commit_message>
<xml_diff>
--- a/LB_Program_Statements.xlsx
+++ b/LB_Program_Statements.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SHREYA\Desktop\LB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2C0851E-707D-4773-B26F-290B8AC85B04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6829921B-F59A-4D9F-B9F5-C78F366B60AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{529304FC-C76E-4A78-91F7-2381E30A6342}"/>
+    <workbookView xWindow="2205" yWindow="2205" windowWidth="21600" windowHeight="11295" xr2:uid="{529304FC-C76E-4A78-91F7-2381E30A6342}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="481" uniqueCount="259">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="487" uniqueCount="262">
   <si>
     <t>Jay Ganesh print in c</t>
   </si>
@@ -958,6 +958,15 @@
     <t>accept number and position to check from user
 do iMask = 0x1
 then iMask &lt;&lt; (iPos - 1)</t>
+  </si>
+  <si>
+    <t>left shift operator using for loop</t>
+  </si>
+  <si>
+    <t>Decimal Hexadecimal table till 1000 decimal</t>
+  </si>
+  <si>
+    <t>Decimal Hexadecimal table till 100 decimal</t>
   </si>
 </sst>
 </file>
@@ -1316,7 +1325,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A099BD82-CF9E-4D41-BD71-1A037607BD64}">
-  <dimension ref="A1:C317"/>
+  <dimension ref="A1:C322"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="93.140625" bestFit="1" customWidth="1"/>
@@ -3245,6 +3254,30 @@
         <v>100</v>
       </c>
     </row>
+    <row r="320" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A320" t="s">
+        <v>261</v>
+      </c>
+      <c r="B320" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="321" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A321" t="s">
+        <v>260</v>
+      </c>
+      <c r="B321" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="322" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A322" t="s">
+        <v>259</v>
+      </c>
+      <c r="B322" t="s">
+        <v>100</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Codes on biwise Operator for toggle the bit position
</commit_message>
<xml_diff>
--- a/LB_Program_Statements.xlsx
+++ b/LB_Program_Statements.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SHREYA\Desktop\LB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6829921B-F59A-4D9F-B9F5-C78F366B60AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE6D9390-B649-464E-ADC1-AAD484BA0855}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2205" yWindow="2205" windowWidth="21600" windowHeight="11295" xr2:uid="{529304FC-C76E-4A78-91F7-2381E30A6342}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="487" uniqueCount="262">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="501" uniqueCount="272">
   <si>
     <t>Jay Ganesh print in c</t>
   </si>
@@ -967,6 +967,41 @@
   </si>
   <si>
     <t>Decimal Hexadecimal table till 100 decimal</t>
+  </si>
+  <si>
+    <t>left shift operator for displaying hexa and decimal
+using for loop = for(iCnt = 1; iCnt &lt;= 33; iCnt++)</t>
+  </si>
+  <si>
+    <t>32 bit ch pusdhe shift zal ki overflow so all become 0 33 wal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0xFFFFFFFF is the largest number in hexa </t>
+  </si>
+  <si>
+    <t>right shift operator for displaying hexa and decimal
+in reverse order  iMask = 0x80000000;</t>
+  </si>
+  <si>
+    <t>right shift operator for displaying hexa and decimal
+ iMask = 0x00000000;</t>
+  </si>
+  <si>
+    <t>Hexadecimal madhe sign unsigned nast</t>
+  </si>
+  <si>
+    <t>toggle the 4th bit</t>
+  </si>
+  <si>
+    <t>iNo ^ iMask  iMask is same with 1 at the position</t>
+  </si>
+  <si>
+    <t>Accept number from user and position of bit
+toggle the position bit</t>
+  </si>
+  <si>
+    <t>Accept number from user and position of bit
+toggle the position bit using a function ToggleBit()</t>
   </si>
 </sst>
 </file>
@@ -1325,7 +1360,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A099BD82-CF9E-4D41-BD71-1A037607BD64}">
-  <dimension ref="A1:C322"/>
+  <dimension ref="A1:C334"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="93.140625" bestFit="1" customWidth="1"/>
@@ -3262,7 +3297,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="321" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A321" t="s">
         <v>260</v>
       </c>
@@ -3270,11 +3305,67 @@
         <v>100</v>
       </c>
     </row>
-    <row r="322" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="322" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A322" t="s">
         <v>259</v>
       </c>
       <c r="B322" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="325" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A325" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="B325" t="s">
+        <v>100</v>
+      </c>
+      <c r="C325" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="326" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A326" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="C326" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="328" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A328" s="1" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="329" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C329" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="330" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A330" s="1" t="s">
+        <v>268</v>
+      </c>
+      <c r="B330" t="s">
+        <v>100</v>
+      </c>
+      <c r="C330" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="333" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A333" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="B333" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="334" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A334" s="1" t="s">
+        <v>271</v>
+      </c>
+      <c r="B334" t="s">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Data structure codes for linkedlist uploded
</commit_message>
<xml_diff>
--- a/LB_Program_Statements.xlsx
+++ b/LB_Program_Statements.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SHREYA\Desktop\LB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE6D9390-B649-464E-ADC1-AAD484BA0855}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC2B9ECF-A30D-46C9-A7C7-1A9AACEEE586}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2205" yWindow="2205" windowWidth="21600" windowHeight="11295" xr2:uid="{529304FC-C76E-4A78-91F7-2381E30A6342}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="501" uniqueCount="272">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="610" uniqueCount="339">
   <si>
     <t>Jay Ganesh print in c</t>
   </si>
@@ -1003,18 +1003,508 @@
     <t>Accept number from user and position of bit
 toggle the position bit using a function ToggleBit()</t>
   </si>
+  <si>
+    <t>Accept number from user and 
+off the bit at 13 th position if its on</t>
+  </si>
+  <si>
+    <t>Accept number from user and 
+off the bit at 23th position if its on</t>
+  </si>
+  <si>
+    <t>iMask = 0xFFBFFFFF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">~ negation operator use 
+UINT iMask = 0xFFFFFFBF; before
+iMask = 40 after </t>
+  </si>
+  <si>
+    <t>toggle position 3 and 7 bit hardcoded positions imask = 0x00000044 for 3 and 7</t>
+  </si>
+  <si>
+    <t>toggle position 12 and 23 bit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">toggle position 21 and 27 bit </t>
+  </si>
+  <si>
+    <t xml:space="preserve">toggle position 9 and 17 bit </t>
+  </si>
+  <si>
+    <t>UINT iMask = 0x04100000;</t>
+  </si>
+  <si>
+    <r>
+      <t>UINT</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFC5C8C6"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF6089B4"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>iMask</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFC5C8C6"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF676867"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>=</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFC5C8C6"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF676867"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>0x</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF6089B4"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>00400800</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFC5C8C6"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>;</t>
+    </r>
+  </si>
+  <si>
+    <t>UINT iMask = 0x00010100;</t>
+  </si>
+  <si>
+    <t>toggle position 3 and 8 bit</t>
+  </si>
+  <si>
+    <r>
+      <t>UINT</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFC5C8C6"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF6089B4"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>iMask</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFC5C8C6"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF676867"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>=</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFC5C8C6"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF676867"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>0x</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF6089B4"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>00000084</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFC5C8C6"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>;</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">toggle position 3 and 8 bit with two masks ored with each other </t>
+  </si>
+  <si>
+    <t>iMask = iMAsk1 | iMask2</t>
+  </si>
+  <si>
+    <t>toggle position 3 and 8 bit with two masks ored with each other by left shift</t>
+  </si>
+  <si>
+    <t>toggle position takin from user bit with two masks
+ ored with each other by left shift</t>
+  </si>
+  <si>
+    <t>structure creation named node for sizeof struct</t>
+  </si>
+  <si>
+    <t>structure creation named node for sizeof struct with paragma pack</t>
+  </si>
+  <si>
+    <t>12 = 4(int) + 8(pointer)</t>
+  </si>
+  <si>
+    <t>16 = 4(int) + 4(padding) + 8(pointer)</t>
+  </si>
+  <si>
+    <t>structure static creation named node and accessing data with dot operator</t>
+  </si>
+  <si>
+    <t>structure static creation named node and creating 2 objects manually
+feels like 2 node linkedlist</t>
+  </si>
+  <si>
+    <t>structure static creation named node and creating 2 objects manually
+Accessing data of seconf node by -&gt; operator</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&amp; gives virtual address not actual physical address </t>
+  </si>
+  <si>
+    <t>structure static creation named node and creating 3 objects manually
+Accessing data of second node by -&gt; operator</t>
+  </si>
+  <si>
+    <t>printf("%d\n",obj1.data);
+    printf("%d\n",obj1.next-&gt;data);
+    printf("%d\n",obj1.next-&gt;next-&gt;data);</t>
+  </si>
+  <si>
+    <t xml:space="preserve">structure static creation named node and creating 3 objects manually
+creating head pointer to first node </t>
+  </si>
+  <si>
+    <t xml:space="preserve">    printf("%d\n",head-&gt;data);
+    printf("%d\n",head-&gt;next-&gt;data);
+    printf("%d\n",head-&gt;next-&gt;next-&gt;data);</t>
+  </si>
+  <si>
+    <t xml:space="preserve">structure static creation named node and creating 3 objects manually
+creating typedef struct node NODE; </t>
+  </si>
+  <si>
+    <t>structure static creation named node and creating 3 objects manually
+typedef struct node NODE;
+typedef struct node * PNODE;</t>
+  </si>
+  <si>
+    <t>manually created 3 objecs of struct node
+traverse the list for display data using temp pointer</t>
+  </si>
+  <si>
+    <t>PNODE temp = head;</t>
+  </si>
+  <si>
+    <t>manually created 3 objecs of struct node
+traverse the list for display data using temp pointer and not while but seuquence</t>
+  </si>
+  <si>
+    <t>manually created 3 objecs of struct node
+traverse the list for display data using temp pointer and while loop</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    while(temp != NULL)
+    {
+        printf("%d\n",temp-&gt;data);   
+        temp = temp-&gt;next;         
+    }</t>
+  </si>
+  <si>
+    <t>manually created 3 objecs of struct node
+traverse the list for counting no of nodes in list</t>
+  </si>
+  <si>
+    <t>dynamically create node object using malloc
+without typedef</t>
+  </si>
+  <si>
+    <t>newn = (struct node *)malloc(sizeof(struct node));</t>
+  </si>
+  <si>
+    <t>count function outside main</t>
+  </si>
+  <si>
+    <r>
+      <t>int</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFC5C8C6"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFCE6700"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>Count</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFC5C8C6"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF9B0000"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>PNODE</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFC5C8C6"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF6089B4"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>temp</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFC5C8C6"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
+  <si>
+    <t>count and display function outside main</t>
+  </si>
+  <si>
+    <t>void Display(PNODE first)</t>
+  </si>
+  <si>
+    <t>full linked list code for
+insert, delete, display, count</t>
+  </si>
+  <si>
+    <t>first is in function and head is in main</t>
+  </si>
+  <si>
+    <t xml:space="preserve">create typedef PPNODE as pointer which holds address of head </t>
+  </si>
+  <si>
+    <t>PNODE head = NULL for avoid runtime accidents</t>
+  </si>
+  <si>
+    <t>create typedef differently</t>
+  </si>
+  <si>
+    <t>typedef struct node 
+{
+    int data;
+    struct node * next;
+}NODE, *PNODE, **PPNODE;</t>
+  </si>
+  <si>
+    <t>create declaration of all functions</t>
+  </si>
+  <si>
+    <t>function declaration without body</t>
+  </si>
+  <si>
+    <t>created function InsertFirst</t>
+  </si>
+  <si>
+    <t>PNODE newn = NULL;        // created pointer which will point to a node
+    newn = (PNODE)malloc(sizeof(NODE));  // created node dynamically</t>
+  </si>
+  <si>
+    <t>InsertFist and Display function function</t>
+  </si>
+  <si>
+    <t xml:space="preserve">beautified Display function with a || around </t>
+  </si>
+  <si>
+    <t xml:space="preserve">count function </t>
+  </si>
+  <si>
+    <t>if(first) == if(first != NULL)</t>
+  </si>
+  <si>
+    <t>if(*first = NULL) is ISSUE</t>
+  </si>
+  <si>
+    <t>if(NULL == *first) == if(first != NULL)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">if(NULL = *first) is ERROR so its a good thing 
+it will be detected while writing code </t>
+  </si>
+  <si>
+    <t>industrial programming practice</t>
+  </si>
+  <si>
+    <t>InsertLast function</t>
+  </si>
+  <si>
+    <t>while(temp-&gt;next != NULL)</t>
+  </si>
+  <si>
+    <t>DeleteLast function
+have 3 conditions empty, 1 node, more</t>
+  </si>
+  <si>
+    <t>DeleteFirst function
+have 3 conditions empty, 1 node, more</t>
+  </si>
+  <si>
+    <t>InsertAtPos function</t>
+  </si>
+  <si>
+    <t>DeleteAtPos function</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFC5C8C6"/>
+      <name val="Courier New"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9B0000"/>
+      <name val="Courier New"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF6089B4"/>
+      <name val="Courier New"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF676867"/>
+      <name val="Courier New"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9A9B99"/>
+      <name val="Courier New"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9872A2"/>
+      <name val="Courier New"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFCE6700"/>
+      <name val="Courier New"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1037,7 +1527,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1045,6 +1535,15 @@
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1360,7 +1859,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A099BD82-CF9E-4D41-BD71-1A037607BD64}">
-  <dimension ref="A1:C334"/>
+  <dimension ref="A1:C384"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="93.140625" bestFit="1" customWidth="1"/>
@@ -3369,7 +3868,423 @@
         <v>100</v>
       </c>
     </row>
+    <row r="338" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A338" s="1" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="339" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A339" s="1" t="s">
+        <v>273</v>
+      </c>
+      <c r="B339" t="s">
+        <v>100</v>
+      </c>
+      <c r="C339" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="342" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A342" s="1" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="343" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A343" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="B343" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="344" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A344" s="1" t="s">
+        <v>279</v>
+      </c>
+      <c r="B344" t="s">
+        <v>100</v>
+      </c>
+      <c r="C344" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="345" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A345" t="s">
+        <v>277</v>
+      </c>
+      <c r="B345" t="s">
+        <v>100</v>
+      </c>
+      <c r="C345" s="4" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="346" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A346" t="s">
+        <v>278</v>
+      </c>
+      <c r="B346" t="s">
+        <v>100</v>
+      </c>
+      <c r="C346" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="347" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A347" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="B347" t="s">
+        <v>100</v>
+      </c>
+      <c r="C347" s="4" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="348" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A348" s="5" t="s">
+        <v>285</v>
+      </c>
+      <c r="B348" t="s">
+        <v>100</v>
+      </c>
+      <c r="C348" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="349" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A349" t="s">
+        <v>287</v>
+      </c>
+      <c r="B349" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="350" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A350" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="B350" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="351" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A351" t="s">
+        <v>289</v>
+      </c>
+      <c r="B351" t="s">
+        <v>100</v>
+      </c>
+      <c r="C351" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="352" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A352" t="s">
+        <v>290</v>
+      </c>
+      <c r="B352" t="s">
+        <v>100</v>
+      </c>
+      <c r="C352" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="353" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A353" t="s">
+        <v>293</v>
+      </c>
+      <c r="B353" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="354" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A354" s="1" t="s">
+        <v>294</v>
+      </c>
+      <c r="B354" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="355" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A355" s="1" t="s">
+        <v>295</v>
+      </c>
+      <c r="B355" t="s">
+        <v>100</v>
+      </c>
+      <c r="C355" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="356" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A356" s="1" t="s">
+        <v>297</v>
+      </c>
+      <c r="B356" t="s">
+        <v>100</v>
+      </c>
+      <c r="C356" s="1" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="357" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A357" s="1" t="s">
+        <v>299</v>
+      </c>
+      <c r="B357" t="s">
+        <v>100</v>
+      </c>
+      <c r="C357" s="1" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="358" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A358" s="1" t="s">
+        <v>301</v>
+      </c>
+      <c r="B358" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="359" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A359" s="1" t="s">
+        <v>302</v>
+      </c>
+      <c r="B359" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="360" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A360" s="1" t="s">
+        <v>303</v>
+      </c>
+      <c r="B360" t="s">
+        <v>100</v>
+      </c>
+      <c r="C360" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="361" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A361" s="1" t="s">
+        <v>305</v>
+      </c>
+      <c r="B361" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="362" spans="1:3" ht="75" x14ac:dyDescent="0.25">
+      <c r="A362" s="1" t="s">
+        <v>306</v>
+      </c>
+      <c r="B362" t="s">
+        <v>100</v>
+      </c>
+      <c r="C362" s="1" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="363" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A363" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="B363" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="364" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A364" s="1" t="s">
+        <v>309</v>
+      </c>
+      <c r="B364" t="s">
+        <v>100</v>
+      </c>
+      <c r="C364" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="365" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A365" s="1" t="s">
+        <v>311</v>
+      </c>
+      <c r="B365" t="s">
+        <v>100</v>
+      </c>
+      <c r="C365" s="6" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="366" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A366" s="1" t="s">
+        <v>313</v>
+      </c>
+      <c r="B366" t="s">
+        <v>100</v>
+      </c>
+      <c r="C366" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="367" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A367" s="1" t="s">
+        <v>315</v>
+      </c>
+      <c r="B367" t="s">
+        <v>100</v>
+      </c>
+      <c r="C367" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="368" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A368" s="5" t="s">
+        <v>317</v>
+      </c>
+      <c r="B368" t="s">
+        <v>100</v>
+      </c>
+      <c r="C368" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="369" spans="1:3" ht="75" x14ac:dyDescent="0.25">
+      <c r="A369" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="B369" t="s">
+        <v>100</v>
+      </c>
+      <c r="C369" s="1" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="370" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A370" s="1" t="s">
+        <v>321</v>
+      </c>
+      <c r="B370" t="s">
+        <v>100</v>
+      </c>
+      <c r="C370" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="371" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A371" s="1" t="s">
+        <v>323</v>
+      </c>
+      <c r="B371" t="s">
+        <v>100</v>
+      </c>
+      <c r="C371" s="1" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="372" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A372" s="1" t="s">
+        <v>325</v>
+      </c>
+      <c r="B372" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="373" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A373" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="B373" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="374" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A374" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="B374" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="375" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A375" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="B375" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="376" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A376" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="B376" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="377" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A377" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="B377" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="378" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A378" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="B378" t="s">
+        <v>100</v>
+      </c>
+      <c r="C378" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="380" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A380" s="5" t="s">
+        <v>333</v>
+      </c>
+      <c r="B380" t="s">
+        <v>100</v>
+      </c>
+      <c r="C380" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="381" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A381" s="1" t="s">
+        <v>336</v>
+      </c>
+      <c r="B381" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="382" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A382" s="1" t="s">
+        <v>335</v>
+      </c>
+      <c r="B382" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="383" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A383" s="1" t="s">
+        <v>337</v>
+      </c>
+      <c r="B383" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="384" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A384" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="B384" t="s">
+        <v>100</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Doubly linear linkedlist code uploded
</commit_message>
<xml_diff>
--- a/LB_Program_Statements.xlsx
+++ b/LB_Program_Statements.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SHREYA\Desktop\LB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC2B9ECF-A30D-46C9-A7C7-1A9AACEEE586}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F221C5A-046B-458D-9E3C-278ED75B96E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2205" yWindow="2205" windowWidth="21600" windowHeight="11295" xr2:uid="{529304FC-C76E-4A78-91F7-2381E30A6342}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="610" uniqueCount="339">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="637" uniqueCount="354">
   <si>
     <t>Jay Ganesh print in c</t>
   </si>
@@ -1450,6 +1450,51 @@
   </si>
   <si>
     <t>DeleteAtPos function</t>
+  </si>
+  <si>
+    <t>Structure creation for Doubly LinkedList</t>
+  </si>
+  <si>
+    <t>3 variables data, next and prev</t>
+  </si>
+  <si>
+    <t>8 function template for DLL</t>
+  </si>
+  <si>
+    <t>InsertFirst function for DLL</t>
+  </si>
+  <si>
+    <t>InsertLast function for DLL</t>
+  </si>
+  <si>
+    <t>(*first)-&gt;prev = newn;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">newn-&gt;prev = temp; </t>
+  </si>
+  <si>
+    <t>Display function for DLL</t>
+  </si>
+  <si>
+    <t>handle 3 conditoons empty 1 node and more</t>
+  </si>
+  <si>
+    <t>DeleteFirst function for DLL</t>
+  </si>
+  <si>
+    <t>DeleteLast function for DLL</t>
+  </si>
+  <si>
+    <t>type 3 while</t>
+  </si>
+  <si>
+    <t>InsertAtPos function for DLL</t>
+  </si>
+  <si>
+    <t>InsertAtPos and DeleteAtPos function half creation for DLL</t>
+  </si>
+  <si>
+    <t>DeleteAtPos function for DLL</t>
   </si>
 </sst>
 </file>
@@ -1859,7 +1904,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A099BD82-CF9E-4D41-BD71-1A037607BD64}">
-  <dimension ref="A1:C384"/>
+  <dimension ref="A1:C395"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="93.140625" bestFit="1" customWidth="1"/>
@@ -4283,6 +4328,109 @@
         <v>100</v>
       </c>
     </row>
+    <row r="385" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A385" s="1" t="s">
+        <v>339</v>
+      </c>
+      <c r="B385" t="s">
+        <v>100</v>
+      </c>
+      <c r="C385" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="386" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A386" s="1" t="s">
+        <v>341</v>
+      </c>
+      <c r="B386" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="387" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A387" s="1" t="s">
+        <v>342</v>
+      </c>
+      <c r="B387" t="s">
+        <v>100</v>
+      </c>
+      <c r="C387" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="388" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A388" s="1" t="s">
+        <v>343</v>
+      </c>
+      <c r="B388" t="s">
+        <v>100</v>
+      </c>
+      <c r="C388" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="389" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A389" s="1" t="s">
+        <v>346</v>
+      </c>
+      <c r="B389" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="390" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A390" s="1" t="s">
+        <v>346</v>
+      </c>
+      <c r="B390" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="391" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A391" s="1" t="s">
+        <v>348</v>
+      </c>
+      <c r="B391" t="s">
+        <v>100</v>
+      </c>
+      <c r="C391" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="392" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A392" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="B392" t="s">
+        <v>100</v>
+      </c>
+      <c r="C392" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="393" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A393" s="1" t="s">
+        <v>352</v>
+      </c>
+      <c r="B393" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="394" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A394" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="B394" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="395" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A395" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="B395" t="s">
+        <v>100</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Linked list code in CPP in OOP approach
</commit_message>
<xml_diff>
--- a/LB_Program_Statements.xlsx
+++ b/LB_Program_Statements.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SHREYA\Desktop\LB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F221C5A-046B-458D-9E3C-278ED75B96E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7489CFA-3CAA-493F-BAA8-D779D2EFFD6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2205" yWindow="2205" windowWidth="21600" windowHeight="11295" xr2:uid="{529304FC-C76E-4A78-91F7-2381E30A6342}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="637" uniqueCount="354">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="673" uniqueCount="373">
   <si>
     <t>Jay Ganesh print in c</t>
   </si>
@@ -1495,6 +1495,72 @@
   </si>
   <si>
     <t>DeleteAtPos function for DLL</t>
+  </si>
+  <si>
+    <t>Singly linear LL Node creation and size of object display in cpp
+acoording to oop node as structure</t>
+  </si>
+  <si>
+    <t>new object created dynamically with new named newn
+and accessed the data with -&gt;</t>
+  </si>
+  <si>
+    <t>cpp</t>
+  </si>
+  <si>
+    <t>class SinglyLL created which has first PNODE</t>
+  </si>
+  <si>
+    <t>class SinglyLL have 2 characteristics and first and iCount
+each time isert called iCount++
+and delete so iCount--</t>
+  </si>
+  <si>
+    <t>so time complexity for while in Count() redused to 0 great</t>
+  </si>
+  <si>
+    <t>first and iCount is public so can be changed in main 
+so not good</t>
+  </si>
+  <si>
+    <t>first and iCount is private 
+so cant be accessed in main so no drawback</t>
+  </si>
+  <si>
+    <t>Count function and 
+all 8 function declaration in class</t>
+  </si>
+  <si>
+    <t>PPNODE is unused so remove</t>
+  </si>
+  <si>
+    <t>all 8 functions are defined in class
+it should be declared in class and defined outside class</t>
+  </si>
+  <si>
+    <t>Display function in cpp</t>
+  </si>
+  <si>
+    <t>InsertFirst function in cpp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Insertlast function </t>
+  </si>
+  <si>
+    <t>while(temp != NULL) is equal to for(i= 1; i&lt;= this-&gt;iCount;i++)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DeleteFirst function </t>
+  </si>
+  <si>
+    <t xml:space="preserve">DeleteLast function </t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsertAtPos function </t>
+  </si>
+  <si>
+    <t>Doubly Linear LinkedList
+all 8 functions are defined for DLL</t>
   </si>
 </sst>
 </file>
@@ -1904,7 +1970,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A099BD82-CF9E-4D41-BD71-1A037607BD64}">
-  <dimension ref="A1:C395"/>
+  <dimension ref="A1:C413"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="93.140625" bestFit="1" customWidth="1"/>
@@ -4431,6 +4497,148 @@
         <v>100</v>
       </c>
     </row>
+    <row r="396" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A396" s="1" t="s">
+        <v>354</v>
+      </c>
+      <c r="B396" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="397" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A397" s="1" t="s">
+        <v>355</v>
+      </c>
+      <c r="B397" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="398" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A398" s="1" t="s">
+        <v>357</v>
+      </c>
+      <c r="B398" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="399" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A399" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="B399" t="s">
+        <v>101</v>
+      </c>
+      <c r="C399" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="400" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A400" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="B400" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="401" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A401" s="1" t="s">
+        <v>361</v>
+      </c>
+      <c r="B401" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="402" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A402" s="1" t="s">
+        <v>362</v>
+      </c>
+      <c r="B402" t="s">
+        <v>101</v>
+      </c>
+      <c r="C402" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="403" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A403" s="1" t="s">
+        <v>364</v>
+      </c>
+      <c r="B403" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="404" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A404" s="1" t="s">
+        <v>365</v>
+      </c>
+      <c r="B404" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="405" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A405" s="1" t="s">
+        <v>366</v>
+      </c>
+      <c r="B405" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="406" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A406" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="B406" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="408" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A408" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="B408" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="409" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A409" s="1" t="s">
+        <v>369</v>
+      </c>
+      <c r="B409" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="410" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A410" s="1" t="s">
+        <v>370</v>
+      </c>
+      <c r="B410" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="411" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A411" s="1" t="s">
+        <v>371</v>
+      </c>
+      <c r="B411" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="412" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A412" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="B412" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="413" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A413" s="1" t="s">
+        <v>372</v>
+      </c>
+      <c r="B413" t="s">
+        <v>101</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Sigly Circular linkedlist in c and Cpp
</commit_message>
<xml_diff>
--- a/LB_Program_Statements.xlsx
+++ b/LB_Program_Statements.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SHREYA\Desktop\LB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B827FE7-311A-4676-A2DE-1C9CF4657AFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBE4C423-6C7B-41D6-88B8-3AE7547643F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2205" yWindow="2205" windowWidth="21600" windowHeight="11295" xr2:uid="{529304FC-C76E-4A78-91F7-2381E30A6342}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{529304FC-C76E-4A78-91F7-2381E30A6342}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="677" uniqueCount="375">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="714" uniqueCount="393">
   <si>
     <t>Jay Ganesh print in c</t>
   </si>
@@ -1568,6 +1568,69 @@
   <si>
     <t>Options for user for operations called Shell creation
 using Switch cases</t>
+  </si>
+  <si>
+    <t>class chya var pan pragma pack can be done as object have padding</t>
+  </si>
+  <si>
+    <t>Singly circulat LinkedList
+8 Function Template</t>
+  </si>
+  <si>
+    <t>Singly circulat LinkedList
+InsertFirst function</t>
+  </si>
+  <si>
+    <t>Singly circulat LinkedList
+InsertLast function</t>
+  </si>
+  <si>
+    <t>(*last)-&gt;next = *first;  imp</t>
+  </si>
+  <si>
+    <t>Display function not checking condition for empty as it is not good</t>
+  </si>
+  <si>
+    <t>Count function</t>
+  </si>
+  <si>
+    <t>Display function with empty LL condition
+if(first == NULL &amp;&amp; last == NULL)</t>
+  </si>
+  <si>
+    <t>Display function with empty LL Issue</t>
+  </si>
+  <si>
+    <t>Display function with empty LL condition 
+if(first != NULL &amp;&amp; last!= NULL)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DeleteFirst function with temp pointer </t>
+  </si>
+  <si>
+    <t xml:space="preserve">DeleteFirst function without temp pointer </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deletelast function </t>
+  </si>
+  <si>
+    <t>need temp for traversal</t>
+  </si>
+  <si>
+    <t>Singly circular Linkedlist
+node and clas creation</t>
+  </si>
+  <si>
+    <t>Singly circular Linkedlist
+all 8 function template</t>
+  </si>
+  <si>
+    <t>SCL Complete
+all singular circular linkedlist</t>
+  </si>
+  <si>
+    <t>SCL 
+Display function and Count Insert first and last</t>
   </si>
 </sst>
 </file>
@@ -1977,7 +2040,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A099BD82-CF9E-4D41-BD71-1A037607BD64}">
-  <dimension ref="A1:C414"/>
+  <dimension ref="A1:C431"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="93.140625" bestFit="1" customWidth="1"/>
@@ -4661,6 +4724,151 @@
       <c r="B414" t="s">
         <v>101</v>
       </c>
+      <c r="C414" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="415" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A415" s="1" t="s">
+        <v>376</v>
+      </c>
+      <c r="B415" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="416" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A416" s="1" t="s">
+        <v>377</v>
+      </c>
+      <c r="B416" t="s">
+        <v>100</v>
+      </c>
+      <c r="C416" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="417" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A417" s="1" t="s">
+        <v>378</v>
+      </c>
+      <c r="B417" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="418" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A418" s="1" t="s">
+        <v>380</v>
+      </c>
+      <c r="B418" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="419" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A419" s="1" t="s">
+        <v>383</v>
+      </c>
+      <c r="B419" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="420" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A420" s="1" t="s">
+        <v>382</v>
+      </c>
+      <c r="B420" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="421" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A421" s="1" t="s">
+        <v>384</v>
+      </c>
+      <c r="B421" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="422" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A422" t="s">
+        <v>381</v>
+      </c>
+      <c r="B422" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="423" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A423" s="1" t="s">
+        <v>385</v>
+      </c>
+      <c r="B423" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="424" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A424" s="1" t="s">
+        <v>386</v>
+      </c>
+      <c r="B424" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="425" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A425" s="1" t="s">
+        <v>387</v>
+      </c>
+      <c r="B425" t="s">
+        <v>100</v>
+      </c>
+      <c r="C425" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="426" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A426" s="1" t="s">
+        <v>337</v>
+      </c>
+      <c r="B426" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="427" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A427" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="B427" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="428" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A428" s="1" t="s">
+        <v>389</v>
+      </c>
+      <c r="B428" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="429" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A429" s="1" t="s">
+        <v>390</v>
+      </c>
+      <c r="B429" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="430" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A430" s="1" t="s">
+        <v>392</v>
+      </c>
+      <c r="B430" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="431" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A431" s="1" t="s">
+        <v>391</v>
+      </c>
+      <c r="B431" t="s">
+        <v>101</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
CVFS functions and structure
</commit_message>
<xml_diff>
--- a/LB_Program_Statements.xlsx
+++ b/LB_Program_Statements.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SHREYA\Desktop\LB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58028DDE-DE19-4166-B0DE-59625D43B7EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83FC2388-C601-4AED-A86F-1BD46315318B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3855" yWindow="3855" windowWidth="21600" windowHeight="11295" xr2:uid="{529304FC-C76E-4A78-91F7-2381E30A6342}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1055" uniqueCount="566">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1065" uniqueCount="571">
   <si>
     <t>Jay Ganesh print in c</t>
   </si>
@@ -2215,6 +2215,21 @@
   <si>
     <t>#define ERR_OPEN -1  
 best industri code all rules</t>
+  </si>
+  <si>
+    <t>CVFS template with macro and header file</t>
+  </si>
+  <si>
+    <t>Structure declaration for CVFS</t>
+  </si>
+  <si>
+    <t>Global variable for cvfs</t>
+  </si>
+  <si>
+    <t>InitialiseUAREA function creation</t>
+  </si>
+  <si>
+    <t>InitialiseSuperBlock Function</t>
   </si>
 </sst>
 </file>
@@ -2644,7 +2659,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A099BD82-CF9E-4D41-BD71-1A037607BD64}">
-  <dimension ref="A1:C608"/>
+  <dimension ref="A1:C613"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="93.140625" bestFit="1" customWidth="1"/>
@@ -6835,6 +6850,46 @@
         <v>100</v>
       </c>
     </row>
+    <row r="609" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A609" t="s">
+        <v>566</v>
+      </c>
+      <c r="B609" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="610" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A610" t="s">
+        <v>567</v>
+      </c>
+      <c r="B610" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="611" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A611" t="s">
+        <v>568</v>
+      </c>
+      <c r="B611" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="612" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A612" t="s">
+        <v>569</v>
+      </c>
+      <c r="B612" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="613" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A613" t="s">
+        <v>570</v>
+      </c>
+      <c r="B613" t="s">
+        <v>100</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
CVFS structure and functions
</commit_message>
<xml_diff>
--- a/LB_Program_Statements.xlsx
+++ b/LB_Program_Statements.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SHREYA\Desktop\LB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83FC2388-C601-4AED-A86F-1BD46315318B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4EBEED5-36C7-4C32-8F1A-7A86B52B8CA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3855" yWindow="3855" windowWidth="21600" windowHeight="11295" xr2:uid="{529304FC-C76E-4A78-91F7-2381E30A6342}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1065" uniqueCount="571">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1116" uniqueCount="594">
   <si>
     <t>Jay Ganesh print in c</t>
   </si>
@@ -2231,12 +2231,248 @@
   <si>
     <t>InitialiseSuperBlock Function</t>
   </si>
+  <si>
+    <t>printf internally calls write system call
+0 - stdin keyboard
+1 - stdout console
+2 - stderr error for console</t>
+  </si>
+  <si>
+    <t>function parameter chsr array with *</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Display file inforamtion </t>
+  </si>
+  <si>
+    <t>copy content from one file to another Issue</t>
+  </si>
+  <si>
+    <t>copy content from one file to another using function</t>
+  </si>
+  <si>
+    <t>CreateDILB try function</t>
+  </si>
+  <si>
+    <t>n node creation with global head</t>
+  </si>
+  <si>
+    <t>n node creation with global head template</t>
+  </si>
+  <si>
+    <t>CreateDILB in CVFS without initialization</t>
+  </si>
+  <si>
+    <t>CreateDILB in CVFS with all initialization to default value</t>
+  </si>
+  <si>
+    <t>StartAuxillaryDataInitialisation() calling in main</t>
+  </si>
+  <si>
+    <t>StartAuxillaryDataInitialisation() with booting information display</t>
+  </si>
+  <si>
+    <t>newn-&gt;FileName[0] = '\0'; can also be used</t>
+  </si>
+  <si>
+    <t xml:space="preserve">input command from user and displya it </t>
+  </si>
+  <si>
+    <t>scanf("%[^'\n']s",str); == fgets(str,sizeof(str),stdin);</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fgets(str,sizeof(str),stdin); use instead of scanf </t>
+  </si>
+  <si>
+    <t>desrination, howmuch, from where  fget</t>
+  </si>
+  <si>
+    <r>
+      <t>scanf</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFC5C8C6"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF9AA83A"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF8080FF"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>%d</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF9AA83A"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF8080FF"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>%d</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF9AA83A"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF8080FF"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>%d</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF9AA83A"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFC5C8C6"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>,</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF676867"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>&amp;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF6089B4"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>i</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFC5C8C6"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>,</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF676867"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>&amp;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF6089B4"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>j</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFC5C8C6"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>,</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF676867"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>&amp;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF6089B4"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>k</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFC5C8C6"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>);</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve"> iRet = printf("jay Ganesh...\n"); printf gives no of char printed so 14 with n</t>
+  </si>
+  <si>
+    <t>iRet = printf("Marvellous\n");</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> iRet = scanf("%d %d %d",&amp;i,&amp;j,&amp;k); scanf returns number of data it accepts so 3</t>
+  </si>
+  <si>
+    <t>sscanf(str,"%s %s %s",Command1,Command2,Command3);</t>
+  </si>
+  <si>
+    <t xml:space="preserve">char Command[4][20] = {{'\0'}}; for 4 words with max 20 characters </t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2300,6 +2536,18 @@
       <name val="Courier New"/>
       <family val="3"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9AA83A"/>
+      <name val="Courier New"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF8080FF"/>
+      <name val="Courier New"/>
+      <family val="3"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -2321,7 +2569,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2344,6 +2592,12 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2659,10 +2913,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A099BD82-CF9E-4D41-BD71-1A037607BD64}">
-  <dimension ref="A1:C613"/>
+  <dimension ref="A1:C630"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="93.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="106.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="69.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -6794,6 +7048,22 @@
         <v>100</v>
       </c>
     </row>
+    <row r="595" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+      <c r="A595" s="1" t="s">
+        <v>571</v>
+      </c>
+      <c r="B595" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="596" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A596" s="1" t="s">
+        <v>558</v>
+      </c>
+      <c r="B596" t="s">
+        <v>100</v>
+      </c>
+    </row>
     <row r="597" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A597" s="1" t="s">
         <v>559</v>
@@ -6810,6 +7080,14 @@
         <v>100</v>
       </c>
     </row>
+    <row r="599" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A599" s="1" t="s">
+        <v>572</v>
+      </c>
+      <c r="B599" t="s">
+        <v>100</v>
+      </c>
+    </row>
     <row r="600" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A600" t="s">
         <v>561</v>
@@ -6826,6 +7104,30 @@
         <v>100</v>
       </c>
     </row>
+    <row r="602" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A602" s="1" t="s">
+        <v>573</v>
+      </c>
+      <c r="B602" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="603" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A603" s="1" t="s">
+        <v>574</v>
+      </c>
+      <c r="B603" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="604" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A604" s="1" t="s">
+        <v>575</v>
+      </c>
+      <c r="B604" t="s">
+        <v>100</v>
+      </c>
+    </row>
     <row r="605" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A605" t="s">
         <v>563</v>
@@ -6834,6 +7136,14 @@
         <v>100</v>
       </c>
     </row>
+    <row r="606" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A606" s="1" t="s">
+        <v>564</v>
+      </c>
+      <c r="B606" t="s">
+        <v>100</v>
+      </c>
+    </row>
     <row r="607" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A607" s="1" t="s">
         <v>565</v>
@@ -6850,7 +7160,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="609" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="609" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A609" t="s">
         <v>566</v>
       </c>
@@ -6858,7 +7168,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="610" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="610" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A610" t="s">
         <v>567</v>
       </c>
@@ -6866,7 +7176,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="611" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="611" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A611" t="s">
         <v>568</v>
       </c>
@@ -6874,7 +7184,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="612" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="612" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A612" t="s">
         <v>569</v>
       </c>
@@ -6882,11 +7192,156 @@
         <v>100</v>
       </c>
     </row>
-    <row r="613" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="613" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A613" t="s">
         <v>570</v>
       </c>
       <c r="B613" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="614" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A614" t="s">
+        <v>576</v>
+      </c>
+      <c r="B614" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="615" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A615" t="s">
+        <v>578</v>
+      </c>
+      <c r="B615" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="616" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A616" t="s">
+        <v>577</v>
+      </c>
+      <c r="B616" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="617" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A617" t="s">
+        <v>579</v>
+      </c>
+      <c r="B617" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="618" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A618" t="s">
+        <v>579</v>
+      </c>
+      <c r="B618" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="619" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A619" t="s">
+        <v>580</v>
+      </c>
+      <c r="B619" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="620" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A620" t="s">
+        <v>581</v>
+      </c>
+      <c r="B620" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="621" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A621" t="s">
+        <v>582</v>
+      </c>
+      <c r="B621" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="622" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A622" t="s">
+        <v>582</v>
+      </c>
+      <c r="B622" t="s">
+        <v>100</v>
+      </c>
+      <c r="C622" t="s">
+        <v>583</v>
+      </c>
+    </row>
+    <row r="623" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A623" t="s">
+        <v>584</v>
+      </c>
+      <c r="B623" t="s">
+        <v>100</v>
+      </c>
+      <c r="C623" t="s">
+        <v>585</v>
+      </c>
+    </row>
+    <row r="624" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A624" t="s">
+        <v>586</v>
+      </c>
+      <c r="B624" t="s">
+        <v>100</v>
+      </c>
+      <c r="C624" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="625" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A625" s="9" t="s">
+        <v>588</v>
+      </c>
+      <c r="B625" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="626" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A626" s="10" t="s">
+        <v>589</v>
+      </c>
+      <c r="B626" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="627" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A627" t="s">
+        <v>590</v>
+      </c>
+      <c r="B627" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="628" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A628" t="s">
+        <v>591</v>
+      </c>
+      <c r="B628" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="629" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A629" t="s">
+        <v>592</v>
+      </c>
+      <c r="B629" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="630" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A630" t="s">
+        <v>593</v>
+      </c>
+      <c r="B630" t="s">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
CVFS project in C
</commit_message>
<xml_diff>
--- a/LB_Program_Statements.xlsx
+++ b/LB_Program_Statements.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SHREYA\Desktop\LB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1108E1D3-5578-4832-B56E-BB098E766FFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD83083D-516F-425F-8694-8DDB48A6B83D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3855" yWindow="3855" windowWidth="21600" windowHeight="11295" xr2:uid="{529304FC-C76E-4A78-91F7-2381E30A6342}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1148" uniqueCount="608">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1150" uniqueCount="609">
   <si>
     <t>Jay Ganesh print in c</t>
   </si>
@@ -2518,6 +2518,9 @@
   </si>
   <si>
     <t>ManPageDisplay and help function</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ls -a function to dsiplay all info of file </t>
   </si>
 </sst>
 </file>
@@ -2965,7 +2968,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A099BD82-CF9E-4D41-BD71-1A037607BD64}">
-  <dimension ref="A1:C646"/>
+  <dimension ref="A1:C647"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="106.140625" bestFit="1" customWidth="1"/>
@@ -7525,6 +7528,14 @@
         <v>100</v>
       </c>
     </row>
+    <row r="647" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A647" t="s">
+        <v>608</v>
+      </c>
+      <c r="B647" t="s">
+        <v>100</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Packing Unpacking project in java
</commit_message>
<xml_diff>
--- a/LB_Program_Statements.xlsx
+++ b/LB_Program_Statements.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SHREYA\Desktop\LB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD83083D-516F-425F-8694-8DDB48A6B83D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{068FBE06-FE5D-4B79-AAC5-497B669BE64C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3855" yWindow="3855" windowWidth="21600" windowHeight="11295" xr2:uid="{529304FC-C76E-4A78-91F7-2381E30A6342}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1150" uniqueCount="609">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1218" uniqueCount="644">
   <si>
     <t>Jay Ganesh print in c</t>
   </si>
@@ -2521,6 +2521,117 @@
   </si>
   <si>
     <t xml:space="preserve">ls -a function to dsiplay all info of file </t>
+  </si>
+  <si>
+    <t>stat file name function to display detaails of specific file</t>
+  </si>
+  <si>
+    <t>unlink function to delete file</t>
+  </si>
+  <si>
+    <t>man page extended</t>
+  </si>
+  <si>
+    <t>write function of file</t>
+  </si>
+  <si>
+    <t>read file content into buffer and show</t>
+  </si>
+  <si>
+    <t>File creation  =with throws</t>
+  </si>
+  <si>
+    <t xml:space="preserve">File creation with try 2 catch </t>
+  </si>
+  <si>
+    <t>File creation Exception</t>
+  </si>
+  <si>
+    <t>exist function</t>
+  </si>
+  <si>
+    <t>File creation if it does not exist</t>
+  </si>
+  <si>
+    <t>File creation if it does not exist with bret variable</t>
+  </si>
+  <si>
+    <t>File creation variable fobj bret outside try so scopr is good</t>
+  </si>
+  <si>
+    <t>File deletion</t>
+  </si>
+  <si>
+    <t>File write which does not exist
+writer will create file not write in it</t>
+  </si>
+  <si>
+    <t xml:space="preserve">because fobj.close not done </t>
+  </si>
+  <si>
+    <t>File write with closing the file in finally</t>
+  </si>
+  <si>
+    <t>File read with char Buffer array from read
+frobj.read(Buffer,3,10);</t>
+  </si>
+  <si>
+    <t>File inbuilt functions like getnmae etc</t>
+  </si>
+  <si>
+    <t>File read bytes its ascii</t>
+  </si>
+  <si>
+    <t>File read typecast to char</t>
+  </si>
+  <si>
+    <t>all files listed file name size and content copied from one folder to another file</t>
+  </si>
+  <si>
+    <t>all files listed content copied from one folder to another file</t>
+  </si>
+  <si>
+    <t>all files listed content copied from one folder to another file
+not implemented</t>
+  </si>
+  <si>
+    <t>from directory all file name and length of files display</t>
+  </si>
+  <si>
+    <t>from directory all file name of files display</t>
+  </si>
+  <si>
+    <t>Directory if present or not</t>
+  </si>
+  <si>
+    <t>Directory check but not file error</t>
+  </si>
+  <si>
+    <t>all files listed file name size and content 
+copied from one folder to another file by sir</t>
+  </si>
+  <si>
+    <t xml:space="preserve">all resources deallocated </t>
+  </si>
+  <si>
+    <t>trim and replaceall double space to single space
+problem with more than 2 spaces</t>
+  </si>
+  <si>
+    <t xml:space="preserve">string input from user </t>
+  </si>
+  <si>
+    <t>split method for tokenization in String array</t>
+  </si>
+  <si>
+    <t>tokenization of a sentence ito words</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tokenization from class StringX </t>
+  </si>
+  <si>
+    <t>void DisplayWords(String str) from class StringX 
+with word length</t>
   </si>
 </sst>
 </file>
@@ -2968,7 +3079,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A099BD82-CF9E-4D41-BD71-1A037607BD64}">
-  <dimension ref="A1:C647"/>
+  <dimension ref="A1:C715"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="106.140625" bestFit="1" customWidth="1"/>
@@ -7536,6 +7647,278 @@
         <v>100</v>
       </c>
     </row>
+    <row r="648" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A648" t="s">
+        <v>609</v>
+      </c>
+    </row>
+    <row r="649" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A649" t="s">
+        <v>610</v>
+      </c>
+      <c r="B649" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="650" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A650" t="s">
+        <v>611</v>
+      </c>
+      <c r="B650" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="651" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A651" t="s">
+        <v>612</v>
+      </c>
+      <c r="B651" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="652" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A652" t="s">
+        <v>613</v>
+      </c>
+      <c r="B652" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="654" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A654" t="s">
+        <v>616</v>
+      </c>
+      <c r="B654" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="655" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A655" t="s">
+        <v>614</v>
+      </c>
+      <c r="B655" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="656" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A656" t="s">
+        <v>615</v>
+      </c>
+      <c r="B656" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="657" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A657" t="s">
+        <v>617</v>
+      </c>
+      <c r="B657" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="658" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A658" t="s">
+        <v>618</v>
+      </c>
+      <c r="B658" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="659" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A659" t="s">
+        <v>619</v>
+      </c>
+      <c r="B659" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="660" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A660" t="s">
+        <v>620</v>
+      </c>
+      <c r="B660" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="661" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A661" t="s">
+        <v>621</v>
+      </c>
+      <c r="B661" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="663" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A663" s="1" t="s">
+        <v>622</v>
+      </c>
+      <c r="B663" t="s">
+        <v>102</v>
+      </c>
+      <c r="C663" t="s">
+        <v>623</v>
+      </c>
+    </row>
+    <row r="665" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A665" t="s">
+        <v>624</v>
+      </c>
+      <c r="B665" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="666" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A666" t="s">
+        <v>627</v>
+      </c>
+      <c r="B666" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="667" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A667" t="s">
+        <v>628</v>
+      </c>
+      <c r="B667" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="670" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A670" s="1" t="s">
+        <v>625</v>
+      </c>
+      <c r="B670" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="671" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A671" t="s">
+        <v>626</v>
+      </c>
+      <c r="B671" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="686" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A686" t="s">
+        <v>635</v>
+      </c>
+      <c r="B686" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="687" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A687" t="s">
+        <v>634</v>
+      </c>
+      <c r="B687" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="688" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A688" t="s">
+        <v>633</v>
+      </c>
+      <c r="B688" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="689" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A689" t="s">
+        <v>632</v>
+      </c>
+      <c r="B689" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="690" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A690" s="1" t="s">
+        <v>631</v>
+      </c>
+      <c r="B690" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="691" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A691" t="s">
+        <v>630</v>
+      </c>
+      <c r="B691" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="692" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A692" t="s">
+        <v>629</v>
+      </c>
+      <c r="B692" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="693" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A693" s="1" t="s">
+        <v>637</v>
+      </c>
+      <c r="B693" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="694" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A694" s="1" t="s">
+        <v>636</v>
+      </c>
+      <c r="B694" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="704" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A704" s="1" t="s">
+        <v>638</v>
+      </c>
+      <c r="B704" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="705" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A705" t="s">
+        <v>639</v>
+      </c>
+      <c r="B705" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="709" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A709" t="s">
+        <v>640</v>
+      </c>
+      <c r="B709" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="712" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A712" t="s">
+        <v>641</v>
+      </c>
+      <c r="B712" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="713" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A713" t="s">
+        <v>642</v>
+      </c>
+      <c r="B713" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="715" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A715" s="1" t="s">
+        <v>643</v>
+      </c>
+      <c r="B715" t="s">
+        <v>102</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
File packer unpacker with Encryption and GUI
</commit_message>
<xml_diff>
--- a/LB_Program_Statements.xlsx
+++ b/LB_Program_Statements.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SHREYA\Desktop\LB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{068FBE06-FE5D-4B79-AAC5-497B669BE64C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7809E7B4-922D-4A3A-B270-26A7CAFBB0CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3855" yWindow="3855" windowWidth="21600" windowHeight="11295" xr2:uid="{529304FC-C76E-4A78-91F7-2381E30A6342}"/>
+    <workbookView xWindow="1560" yWindow="1560" windowWidth="21600" windowHeight="11295" xr2:uid="{529304FC-C76E-4A78-91F7-2381E30A6342}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1218" uniqueCount="644">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1222" uniqueCount="646">
   <si>
     <t>Jay Ganesh print in c</t>
   </si>
@@ -2632,6 +2632,12 @@
   <si>
     <t>void DisplayWords(String str) from class StringX 
 with word length</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unpacking all files from a packed file code </t>
+  </si>
+  <si>
+    <t>Final packing code</t>
   </si>
 </sst>
 </file>
@@ -3079,7 +3085,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A099BD82-CF9E-4D41-BD71-1A037607BD64}">
-  <dimension ref="A1:C715"/>
+  <dimension ref="A1:C733"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="106.140625" bestFit="1" customWidth="1"/>
@@ -7919,6 +7925,22 @@
         <v>102</v>
       </c>
     </row>
+    <row r="728" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A728" t="s">
+        <v>645</v>
+      </c>
+      <c r="B728" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="733" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A733" t="s">
+        <v>644</v>
+      </c>
+      <c r="B733" t="s">
+        <v>102</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>